<commit_message>
OCR and visual extraction added
</commit_message>
<xml_diff>
--- a/lubrication_tables.xlsx
+++ b/lubrication_tables.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Table 6" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="CI-4 Hardness" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ISO VG 10" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fig 1 Temperatures" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1375,4 +1376,128 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fig. 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0 C</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>visual fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fig. 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>33 C</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fig. 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>99 C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fig. 1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>218 C</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>